<commit_message>
Update manage movie screen
</commit_message>
<xml_diff>
--- a/src/front-end/public/templates/MovieList-Template.xlsx
+++ b/src/front-end/public/templates/MovieList-Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Movie Title</t>
   </si>
@@ -38,6 +38,42 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Roboto"/>
+        <color rgb="FF000000"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t>Detective Conan: One-Eyed Flashback</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Roboto"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve"> (2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>As police inspector Yamato Kansuke pursues a certain man in the snowy mountains of Nagano, a shadow suddenly appears in his field of vision. While he's distracted, a rifle bullet fired by someone grazes his left eye and causes an avalanche accompanied by a roar. Ten months later, Kansuke, having miraculously survived the avalanche, receives a report that a researcher at the Nobeyama National Astronomical Observatory has been attacked.As police inspector Yamato Kansuke pursues a certain man in the snowy mountains of Nagano, a shadow suddenly appears in his field of vision. While he's distracted, a rifle bullet fired by someone grazes his left eye and causes an avalanche accompanied by a roar. Ten months later, Kansuke, having miraculously survived the avalanche, receives a report that a researcher at the Nobeyama National Astronomical Observatory has been attacked.</t>
+  </si>
+  <si>
+    <t>Animation, Action, Mystery, Crime</t>
+  </si>
+  <si>
+    <t>PG12</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7CSxbEaOb-4</t>
+  </si>
+  <si>
+    <t>https://www.themoviedb.org/t/p/w600_and_h900_bestv2/1wl6eAHbIDSz61tGwYTOKlSRvZb.jpg</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
 </sst>
 </file>
@@ -47,7 +83,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/MM/yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -59,13 +95,45 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -248,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -261,70 +329,88 @@
     <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="3" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="7" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="7" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
     <xf borderId="8" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="12" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="12" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -653,169 +739,187 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="9"/>
+      <c r="A2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6">
+        <v>45765.0</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="8">
+        <v>120.0</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="14"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4">
-      <c r="A4" s="15"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="19"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="24"/>
     </row>
     <row r="5">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="14"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="19"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="24"/>
     </row>
     <row r="7">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="14"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="24"/>
     </row>
     <row r="9">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="14"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10">
-      <c r="A10" s="15"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="19"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="24"/>
     </row>
     <row r="11">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="14"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="19"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="24"/>
     </row>
     <row r="13">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="14"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="19"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="24"/>
     </row>
     <row r="15">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="14"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="19"/>
     </row>
     <row r="16">
-      <c r="A16" s="22"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="25"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="31"/>
     </row>
   </sheetData>
   <dataValidations>
@@ -827,9 +931,13 @@
     </dataValidation>
     <dataValidation allowBlank="1" showDropDown="1" sqref="A2:B15 D2:D15 F2:I15"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="G2"/>
+    <hyperlink r:id="rId2" ref="H2"/>
+  </hyperlinks>
+  <drawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>